<commit_message>
Automatiza 81 arquivo(s) de processos no backend
</commit_message>
<xml_diff>
--- a/planilhas/LISTA DE PROCESSO PG BACKLIGHT MOD 5.xlsx
+++ b/planilhas/LISTA DE PROCESSO PG BACKLIGHT MOD 5.xlsx
@@ -62,10 +62,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -345,7 +344,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F35"/>
+  <dimension ref="A1:F55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -404,14 +403,14 @@
           <t>0,75 Nest 1</t>
         </is>
       </c>
-      <c r="D2" s="3">
+      <c r="D2" s="2">
         <f>E2/19</f>
         <v/>
       </c>
       <c r="E2" t="n">
         <v>2</v>
       </c>
-      <c r="F2" s="4" t="inlineStr">
+      <c r="F2" s="3" t="inlineStr">
         <is>
           <t>001810</t>
         </is>
@@ -433,14 +432,14 @@
           <t>0,75 Nest 2</t>
         </is>
       </c>
-      <c r="D3" s="3">
+      <c r="D3" s="2">
         <f>E3/19</f>
         <v/>
       </c>
       <c r="E3" t="n">
         <v>1</v>
       </c>
-      <c r="F3" s="4" t="inlineStr">
+      <c r="F3" s="3" t="inlineStr">
         <is>
           <t>001811</t>
         </is>
@@ -462,14 +461,14 @@
           <t>0,75 Nest 3</t>
         </is>
       </c>
-      <c r="D4" s="3">
+      <c r="D4" s="2">
         <f>E4/19</f>
         <v/>
       </c>
       <c r="E4" t="n">
         <v>11</v>
       </c>
-      <c r="F4" s="4" t="inlineStr">
+      <c r="F4" s="3" t="inlineStr">
         <is>
           <t>001812</t>
         </is>
@@ -491,14 +490,14 @@
           <t>0,75 Nest 4</t>
         </is>
       </c>
-      <c r="D5" s="3">
+      <c r="D5" s="2">
         <f>E5/19</f>
         <v/>
       </c>
       <c r="E5" t="n">
         <v>3</v>
       </c>
-      <c r="F5" s="4" t="inlineStr">
+      <c r="F5" s="3" t="inlineStr">
         <is>
           <t>001813</t>
         </is>
@@ -520,14 +519,14 @@
           <t>0,75 Nest 5</t>
         </is>
       </c>
-      <c r="D6" s="3">
+      <c r="D6" s="2">
         <f>E6/19</f>
         <v/>
       </c>
       <c r="E6" t="n">
         <v>4</v>
       </c>
-      <c r="F6" s="4" t="inlineStr">
+      <c r="F6" s="3" t="inlineStr">
         <is>
           <t>001814</t>
         </is>
@@ -549,14 +548,14 @@
           <t>0,75 Nest 6</t>
         </is>
       </c>
-      <c r="D7" s="3">
+      <c r="D7" s="2">
         <f>E7/19</f>
         <v/>
       </c>
       <c r="E7" t="n">
         <v>1</v>
       </c>
-      <c r="F7" s="4" t="inlineStr">
+      <c r="F7" s="3" t="inlineStr">
         <is>
           <t>001815</t>
         </is>
@@ -578,14 +577,14 @@
           <t>0,75 Nest 7</t>
         </is>
       </c>
-      <c r="D8" s="3">
+      <c r="D8" s="2">
         <f>E8/19</f>
         <v/>
       </c>
       <c r="E8" t="n">
         <v>8</v>
       </c>
-      <c r="F8" s="4" t="inlineStr">
+      <c r="F8" s="3" t="inlineStr">
         <is>
           <t>001816</t>
         </is>
@@ -607,14 +606,14 @@
           <t>0,75 Nest 8</t>
         </is>
       </c>
-      <c r="D9" s="3">
+      <c r="D9" s="2">
         <f>E9/19</f>
         <v/>
       </c>
       <c r="E9" t="n">
         <v>2</v>
       </c>
-      <c r="F9" s="4" t="inlineStr">
+      <c r="F9" s="3" t="inlineStr">
         <is>
           <t>001817</t>
         </is>
@@ -636,14 +635,14 @@
           <t>0,75 Nest 9</t>
         </is>
       </c>
-      <c r="D10" s="3">
+      <c r="D10" s="2">
         <f>E10/19</f>
         <v/>
       </c>
       <c r="E10" t="n">
         <v>2</v>
       </c>
-      <c r="F10" s="4" t="inlineStr">
+      <c r="F10" s="3" t="inlineStr">
         <is>
           <t>001818</t>
         </is>
@@ -665,14 +664,14 @@
           <t>0,75 Nest 10</t>
         </is>
       </c>
-      <c r="D11" s="3">
+      <c r="D11" s="2">
         <f>E11/19</f>
         <v/>
       </c>
       <c r="E11" t="n">
         <v>1</v>
       </c>
-      <c r="F11" s="4" t="inlineStr">
+      <c r="F11" s="3" t="inlineStr">
         <is>
           <t>001819</t>
         </is>
@@ -694,14 +693,14 @@
           <t>0,9 Nest 1</t>
         </is>
       </c>
-      <c r="D12" s="3">
+      <c r="D12" s="2">
         <f>E12/19</f>
         <v/>
       </c>
       <c r="E12" t="n">
         <v>12</v>
       </c>
-      <c r="F12" s="4" t="inlineStr">
+      <c r="F12" s="3" t="inlineStr">
         <is>
           <t>001820</t>
         </is>
@@ -723,14 +722,14 @@
           <t>0,9 Nest 2</t>
         </is>
       </c>
-      <c r="D13" s="3">
+      <c r="D13" s="2">
         <f>E13/19</f>
         <v/>
       </c>
       <c r="E13" t="n">
         <v>24</v>
       </c>
-      <c r="F13" s="4" t="inlineStr">
+      <c r="F13" s="3" t="inlineStr">
         <is>
           <t>001821</t>
         </is>
@@ -752,14 +751,14 @@
           <t>0,9 Nest 3</t>
         </is>
       </c>
-      <c r="D14" s="3">
+      <c r="D14" s="2">
         <f>E14/19</f>
         <v/>
       </c>
       <c r="E14" t="n">
         <v>35</v>
       </c>
-      <c r="F14" s="4" t="inlineStr">
+      <c r="F14" s="3" t="inlineStr">
         <is>
           <t>001822</t>
         </is>
@@ -781,14 +780,14 @@
           <t>0,9 Nest 4</t>
         </is>
       </c>
-      <c r="D15" s="3">
+      <c r="D15" s="2">
         <f>E15/19</f>
         <v/>
       </c>
       <c r="E15" t="n">
         <v>1</v>
       </c>
-      <c r="F15" s="4" t="inlineStr">
+      <c r="F15" s="3" t="inlineStr">
         <is>
           <t>001823</t>
         </is>
@@ -816,7 +815,7 @@
       <c r="E16" t="n">
         <v>19</v>
       </c>
-      <c r="F16" s="4" t="inlineStr">
+      <c r="F16" s="3" t="inlineStr">
         <is>
           <t>001824</t>
         </is>
@@ -844,7 +843,7 @@
       <c r="E17" t="n">
         <v>19</v>
       </c>
-      <c r="F17" s="4" t="inlineStr">
+      <c r="F17" s="3" t="inlineStr">
         <is>
           <t>001825</t>
         </is>
@@ -872,7 +871,7 @@
       <c r="E18" t="n">
         <v>76</v>
       </c>
-      <c r="F18" s="4" t="inlineStr">
+      <c r="F18" s="3" t="inlineStr">
         <is>
           <t>001826</t>
         </is>
@@ -900,7 +899,7 @@
       <c r="E19" t="n">
         <v>152</v>
       </c>
-      <c r="F19" s="4" t="inlineStr">
+      <c r="F19" s="3" t="inlineStr">
         <is>
           <t>001827</t>
         </is>
@@ -928,7 +927,7 @@
       <c r="E20" t="n">
         <v>76</v>
       </c>
-      <c r="F20" s="4" t="inlineStr">
+      <c r="F20" s="3" t="inlineStr">
         <is>
           <t>001828</t>
         </is>
@@ -956,7 +955,7 @@
       <c r="E21" t="n">
         <v>76</v>
       </c>
-      <c r="F21" s="4" t="inlineStr">
+      <c r="F21" s="3" t="inlineStr">
         <is>
           <t>001829</t>
         </is>
@@ -984,7 +983,7 @@
       <c r="E22" t="n">
         <v>57</v>
       </c>
-      <c r="F22" s="4" t="inlineStr">
+      <c r="F22" s="3" t="inlineStr">
         <is>
           <t>001830</t>
         </is>
@@ -1012,7 +1011,7 @@
       <c r="E23" t="n">
         <v>19</v>
       </c>
-      <c r="F23" s="4" t="inlineStr">
+      <c r="F23" s="3" t="inlineStr">
         <is>
           <t>001831</t>
         </is>
@@ -1040,7 +1039,7 @@
       <c r="E24" t="n">
         <v>76</v>
       </c>
-      <c r="F24" s="4" t="inlineStr">
+      <c r="F24" s="3" t="inlineStr">
         <is>
           <t>001832</t>
         </is>
@@ -1068,7 +1067,7 @@
       <c r="E25" t="n">
         <v>38</v>
       </c>
-      <c r="F25" s="4" t="inlineStr">
+      <c r="F25" s="3" t="inlineStr">
         <is>
           <t>001833</t>
         </is>
@@ -1096,7 +1095,7 @@
       <c r="E26" t="n">
         <v>38</v>
       </c>
-      <c r="F26" s="4" t="inlineStr">
+      <c r="F26" s="3" t="inlineStr">
         <is>
           <t>001834</t>
         </is>
@@ -1124,7 +1123,7 @@
       <c r="E27" t="n">
         <v>114</v>
       </c>
-      <c r="F27" s="4" t="inlineStr">
+      <c r="F27" s="3" t="inlineStr">
         <is>
           <t>001835</t>
         </is>
@@ -1152,7 +1151,7 @@
       <c r="E28" t="n">
         <v>76</v>
       </c>
-      <c r="F28" s="4" t="inlineStr">
+      <c r="F28" s="3" t="inlineStr">
         <is>
           <t>001836</t>
         </is>
@@ -1180,7 +1179,7 @@
       <c r="E29" t="n">
         <v>152</v>
       </c>
-      <c r="F29" s="4" t="inlineStr">
+      <c r="F29" s="3" t="inlineStr">
         <is>
           <t>001837</t>
         </is>
@@ -1208,7 +1207,7 @@
       <c r="E30" t="n">
         <v>152</v>
       </c>
-      <c r="F30" s="4" t="inlineStr">
+      <c r="F30" s="3" t="inlineStr">
         <is>
           <t>001838</t>
         </is>
@@ -1236,7 +1235,7 @@
       <c r="E31" t="n">
         <v>19</v>
       </c>
-      <c r="F31" s="4" t="inlineStr">
+      <c r="F31" s="3" t="inlineStr">
         <is>
           <t>001839</t>
         </is>
@@ -1264,7 +1263,7 @@
       <c r="E32" t="n">
         <v>57</v>
       </c>
-      <c r="F32" s="4" t="inlineStr">
+      <c r="F32" s="3" t="inlineStr">
         <is>
           <t>001840</t>
         </is>
@@ -1292,7 +1291,7 @@
       <c r="E33" t="n">
         <v>19</v>
       </c>
-      <c r="F33" s="4" t="inlineStr">
+      <c r="F33" s="3" t="inlineStr">
         <is>
           <t>001841</t>
         </is>
@@ -1320,7 +1319,7 @@
       <c r="E34" t="n">
         <v>76</v>
       </c>
-      <c r="F34" s="4" t="inlineStr">
+      <c r="F34" s="3" t="inlineStr">
         <is>
           <t>001842</t>
         </is>
@@ -1348,9 +1347,569 @@
       <c r="E35" t="n">
         <v>38</v>
       </c>
-      <c r="F35" s="4" t="inlineStr">
+      <c r="F35" s="3" t="inlineStr">
         <is>
           <t>001843</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>PG BACKLIGHT MOD 5</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Solda Mig</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Quadro do Corpo LE</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>19</v>
+      </c>
+      <c r="E36" t="n">
+        <v>19</v>
+      </c>
+      <c r="F36" s="3" t="inlineStr">
+        <is>
+          <t>001844</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>PG BACKLIGHT MOD 5</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Solda Mig</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Quadro do Corpo LD</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>19</v>
+      </c>
+      <c r="E37" t="n">
+        <v>19</v>
+      </c>
+      <c r="F37" s="3" t="inlineStr">
+        <is>
+          <t>001845</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>PG BACKLIGHT MOD 5</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Solda Mig</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Quadro Testeira</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>19</v>
+      </c>
+      <c r="E38" t="n">
+        <v>38</v>
+      </c>
+      <c r="F38" s="3" t="inlineStr">
+        <is>
+          <t>001846</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>PG BACKLIGHT MOD 5</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Solda Mig</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Testeira</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>19</v>
+      </c>
+      <c r="E39" t="n">
+        <v>19</v>
+      </c>
+      <c r="F39" s="3" t="inlineStr">
+        <is>
+          <t>001847</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>PG BACKLIGHT MOD 5</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Solda Mig</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Canaleta Testeira</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>19</v>
+      </c>
+      <c r="E40" t="n">
+        <v>19</v>
+      </c>
+      <c r="F40" s="3" t="inlineStr">
+        <is>
+          <t>001848</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>PG BACKLIGHT MOD 5</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Solda Mig</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Corpo Central</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>19</v>
+      </c>
+      <c r="E41" t="n">
+        <v>19</v>
+      </c>
+      <c r="F41" s="3" t="inlineStr">
+        <is>
+          <t>001849</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>PG BACKLIGHT MOD 5</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Solda Mig</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Trava Corpo Central</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>19</v>
+      </c>
+      <c r="E42" t="n">
+        <v>19</v>
+      </c>
+      <c r="F42" s="3" t="inlineStr">
+        <is>
+          <t>001850</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>PG BACKLIGHT MOD 5</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Solda Mig</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Estrutura Lat Esq</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>19</v>
+      </c>
+      <c r="E43" t="n">
+        <v>19</v>
+      </c>
+      <c r="F43" s="3" t="inlineStr">
+        <is>
+          <t>001851</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>PG BACKLIGHT MOD 5</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Solda Mig</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Estrutura Lat Dir</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>19</v>
+      </c>
+      <c r="E44" t="n">
+        <v>19</v>
+      </c>
+      <c r="F44" s="3" t="inlineStr">
+        <is>
+          <t>001852</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>PG BACKLIGHT MOD 5</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Solda Mig</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Cruzeta</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>19</v>
+      </c>
+      <c r="E45" t="n">
+        <v>38</v>
+      </c>
+      <c r="F45" s="3" t="inlineStr">
+        <is>
+          <t>001853</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>PG BACKLIGHT MOD 5</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Solda Mig</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Parachoque</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>19</v>
+      </c>
+      <c r="E46" t="n">
+        <v>38</v>
+      </c>
+      <c r="F46" s="3" t="inlineStr">
+        <is>
+          <t>001854</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>PG BACKLIGHT MOD 5</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Solda Mig</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Chapa do rodizio corpo lateral</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>19</v>
+      </c>
+      <c r="E47" t="n">
+        <v>38</v>
+      </c>
+      <c r="F47" s="3" t="inlineStr">
+        <is>
+          <t>001855</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>PG BACKLIGHT MOD 5</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Solda Mig</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Bdj Maior Lateral</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>19</v>
+      </c>
+      <c r="E48" t="n">
+        <v>152</v>
+      </c>
+      <c r="F48" s="3" t="inlineStr">
+        <is>
+          <t>001856</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>PG BACKLIGHT MOD 5</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Solda Mig</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Arame na Bdj Maior Lat</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>19</v>
+      </c>
+      <c r="E49" t="n">
+        <v>152</v>
+      </c>
+      <c r="F49" s="3" t="inlineStr">
+        <is>
+          <t>001857</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>PG BACKLIGHT MOD 5</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Solda Mig</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Bdj Menor Lateral</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>19</v>
+      </c>
+      <c r="E50" t="n">
+        <v>76</v>
+      </c>
+      <c r="F50" s="3" t="inlineStr">
+        <is>
+          <t>001858</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>PG BACKLIGHT MOD 5</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Solda Mig</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Arame na Bdj Menor Lat</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>19</v>
+      </c>
+      <c r="E51" t="n">
+        <v>76</v>
+      </c>
+      <c r="F51" s="3" t="inlineStr">
+        <is>
+          <t>001859</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>PG BACKLIGHT MOD 5</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Solda Mig</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Bdj Central</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>19</v>
+      </c>
+      <c r="E52" t="n">
+        <v>57</v>
+      </c>
+      <c r="F52" s="3" t="inlineStr">
+        <is>
+          <t>001860</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>PG BACKLIGHT MOD 5</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Solda Mig</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Arame na Bdj Central</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>19</v>
+      </c>
+      <c r="E53" t="n">
+        <v>57</v>
+      </c>
+      <c r="F53" s="3" t="inlineStr">
+        <is>
+          <t>001861</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>PG BACKLIGHT MOD 5</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Solda Mig</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Tubo Curvo Arte Direita</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
+        <v>19</v>
+      </c>
+      <c r="E54" t="n">
+        <v>19</v>
+      </c>
+      <c r="F54" s="3" t="inlineStr">
+        <is>
+          <t>001862</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>PG BACKLIGHT MOD 5</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Solda Mig</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Tubo Curvo Arte Esquerda</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>19</v>
+      </c>
+      <c r="E55" t="n">
+        <v>19</v>
+      </c>
+      <c r="F55" s="3" t="inlineStr">
+        <is>
+          <t>001863</t>
         </is>
       </c>
     </row>

</xml_diff>